<commit_message>
Láminas 8 y 9: Giordano de Georgetown (Meade) y Cano de Kingston Lacy (Bankes)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SBA5XgFAtM5RV8Xy37Ayvq
</commit_message>
<xml_diff>
--- a/control/control_derechos_laminas_20261024.xlsx
+++ b/control/control_derechos_laminas_20261024.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -801,6 +801,88 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>giordano</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Luca Giordano, La vocación de San Mateo (c. 1685)</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Georgetown University Art Collection, Washington (comprado a Martha Meade, 1860)</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>https://library.georgetown.edu/special-collections/art/guac/Giordano</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="n"/>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Condiciones de Georgetown University Library</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>enlazar</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>https://jjr2025.github.io/De_Cadiz_a_Nueva_York/laminas/#giordano</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>cano_nino</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Atribuido a Alonso Cano, El Niño Jesús dormido (c. 1652)</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Kingston Lacy, The Bankes Collection, National Trust (NT 1257133)</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>https://www.nationaltrustcollections.org.uk/object/1257133</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="n"/>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>© National Trust Images</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>enlazar</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>https://jjr2025.github.io/De_Cadiz_a_Nueva_York/laminas/#cano_nino</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
@@ -815,6 +897,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" location="abanico" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" location="resurreccion" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" location="giordano" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" location="cano_nino" r:id="rId16"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Lámina 4: ficha de Sotheby's 2004, lote 53 (Inza)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SBA5XgFAtM5RV8Xy37Ayvq
</commit_message>
<xml_diff>
--- a/control/control_derechos_laminas_20261024.xlsx
+++ b/control/control_derechos_laminas_20261024.xlsx
@@ -657,10 +657,14 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Colección particular</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="n"/>
+          <t>Colección particular. Sotheby's Nueva York, Arcade Fine Arts, 2004, lote 53; 98 × 72,8 cm</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sothebys.com/en/auctions/ecatalogue/2004/arcade-fine-arts-old-master-to-contemporary-n01743/lot.53.html</t>
+        </is>
+      </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
           <t>inza_sothebys.jpg</t>
@@ -891,16 +895,17 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" location="cano" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" location="murillo" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" location="inza" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" location="rufina" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" location="abanico" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" location="resurreccion" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" location="giordano" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" location="cano_nino" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" location="inza" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" location="rufina" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" location="abanico" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" location="resurreccion" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" location="giordano" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" location="cano_nino" r:id="rId17"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Lámina 5: fecha según la Fundación Focus y contacto para cesión de imágenes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SBA5XgFAtM5RV8Xy37Ayvq
</commit_message>
<xml_diff>
--- a/control/control_derechos_laminas_20261024.xlsx
+++ b/control/control_derechos_laminas_20261024.xlsx
@@ -697,7 +697,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Velázquez, Santa Rufina (c. 1632-1634)</t>
+          <t>Velázquez, Santa Rufina (1629-1632)</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -713,7 +713,7 @@
       <c r="F6" s="3" t="n"/>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Pedir autorización a Focus</t>
+          <t>Pedir autorización a Focus (Cesión de imágenes; focus@fundacionfocus.com)</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Lámina 6: ficha del Louvre (RF 1132)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SBA5XgFAtM5RV8Xy37Ayvq
</commit_message>
<xml_diff>
--- a/control/control_derechos_laminas_20261024.xlsx
+++ b/control/control_derechos_laminas_20261024.xlsx
@@ -743,18 +743,18 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Musée du Louvre, París</t>
+          <t>Musée du Louvre, París (RF 1132), comprado en la venta Kums, Amberes, 1898; 103 × 84,5 cm</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>https://fundaciongoyaenaragon.es/obra/mujer-joven-con-abanico/311</t>
+          <t>https://collections.louvre.fr/ark:/53355/cl010064756</t>
         </is>
       </c>
       <c r="F7" s="3" t="n"/>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Condiciones del Louvre / GrandPalaisRmn</t>
+          <t>Condiciones generales de uso del Louvre (descarga tras aceptarlas)</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Lámina 7: lote 680 de Templum (Resurrección)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SBA5XgFAtM5RV8Xy37Ayvq
</commit_message>
<xml_diff>
--- a/control/control_derechos_laminas_20261024.xlsx
+++ b/control/control_derechos_laminas_20261024.xlsx
@@ -784,14 +784,18 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>En venta en 1stDibs</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="n"/>
+          <t>Templum Fine Art Auctions, Madrid, subasta 297, lote 680 («Escuela italiana»); hoy en venta en 1stDibs</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>https://templumauctions.com/auction/297-gran-subasta-de-es/lot-680-escuela-italiana/</t>
+        </is>
+      </c>
       <c r="F8" s="3" t="n"/>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Foto del anunciante</t>
+          <t>Foto de la casa de subastas</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
@@ -901,11 +905,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" location="rufina" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" location="abanico" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" location="resurreccion" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" location="giordano" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" location="cano_nino" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" location="resurreccion" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" location="giordano" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" location="cano_nino" r:id="rId18"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Láminas: imágenes normalizadas (lamina_NN_id.jpg, 1800 px) y publicadas las de dominio público (Met, LACMA, Inza)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SBA5XgFAtM5RV8Xy37Ayvq
</commit_message>
<xml_diff>
--- a/control/control_derechos_laminas_20261024.xlsx
+++ b/control/control_derechos_laminas_20261024.xlsx
@@ -536,7 +536,7 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>goya_met_06289.jpg</t>
+          <t>lamina_01_goya.jpg</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
@@ -579,7 +579,11 @@
           <t>https://hispanicsociety.emuseum.com/objects/963/portrait-of-an-ecclesiastic</t>
         </is>
       </c>
-      <c r="F3" s="3" t="n"/>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>lamina_02_cano.jpg</t>
+        </is>
+      </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Por confirmar condiciones de la Hispanic Society</t>
@@ -622,7 +626,7 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>murillo_lacma_M83168.jpg</t>
+          <t>lamina_03_murillo.jpg</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -667,7 +671,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>inza_sothebys.jpg</t>
+          <t>lamina_04_inza.jpg</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -710,7 +714,11 @@
           <t>https://fundacionfocus.es/centro-velazquez-ant/santa-rufina/</t>
         </is>
       </c>
-      <c r="F6" s="3" t="n"/>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>lamina_05_rufina.jpg</t>
+        </is>
+      </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
           <t>Pedir autorización a Focus (Cesión de imágenes; focus@fundacionfocus.com)</t>
@@ -751,7 +759,11 @@
           <t>https://collections.louvre.fr/ark:/53355/cl010064756</t>
         </is>
       </c>
-      <c r="F7" s="3" t="n"/>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>lamina_06_abanico.jpg</t>
+        </is>
+      </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
           <t>Condiciones generales de uso del Louvre (descarga tras aceptarlas)</t>
@@ -792,7 +804,11 @@
           <t>https://templumauctions.com/auction/297-gran-subasta-de-es/lot-680-escuela-italiana/</t>
         </is>
       </c>
-      <c r="F8" s="3" t="n"/>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>lamina_07_resurreccion.jpg</t>
+        </is>
+      </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
           <t>Foto de la casa de subastas</t>
@@ -833,7 +849,11 @@
           <t>https://library.georgetown.edu/special-collections/art/guac/Giordano</t>
         </is>
       </c>
-      <c r="F9" s="3" t="n"/>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>lamina_08_giordano.jpg</t>
+        </is>
+      </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
           <t>Condiciones de Georgetown University Library</t>
@@ -874,7 +894,11 @@
           <t>https://www.nationaltrustcollections.org.uk/object/1257133</t>
         </is>
       </c>
-      <c r="F10" s="3" t="n"/>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>lamina_09_cano_nino.jpg</t>
+        </is>
+      </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
           <t>© National Trust Images</t>

</xml_diff>